<commit_message>
After the IDMA oral exam
</commit_message>
<xml_diff>
--- a/ExamOral_2026/GradingSheet_IDMA26_OralExam_260624_260629.xlsx
+++ b/ExamOral_2026/GradingSheet_IDMA26_OralExam_260624_260629.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Teaching\IDMA26\ExamOral_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF966F8-9AF8-4AE3-9F85-87D1C77CDA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97BFD74-6C3A-4BFE-A4CB-83AFF7908E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="20057" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grading sheet" sheetId="1" r:id="rId1"/>
@@ -737,7 +737,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -762,12 +762,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1190,23 +1184,23 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A12" s="9">
         <v>0.375</v>
       </c>
@@ -1216,17 +1210,17 @@
       <c r="C12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="9">
         <v>0.39583333333333331</v>
       </c>
@@ -1236,17 +1230,17 @@
       <c r="C13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
       <c r="L13" s="8"/>
     </row>
-    <row r="14" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="9">
         <v>0.41666666666666669</v>
       </c>
@@ -1256,17 +1250,17 @@
       <c r="C14" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
       <c r="L14" s="8"/>
     </row>
-    <row r="15" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15" s="9">
         <v>0.4375</v>
       </c>
@@ -1276,17 +1270,17 @@
       <c r="C15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" spans="1:15" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:15" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A16" s="9">
         <v>0.45833333333333298</v>
       </c>
@@ -1296,17 +1290,17 @@
       <c r="C16" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
       <c r="L16" s="8"/>
     </row>
-    <row r="17" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="9">
         <v>0.47916666666666702</v>
       </c>
@@ -1316,33 +1310,33 @@
       <c r="C17" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
       <c r="L17" s="8"/>
     </row>
-    <row r="18" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A18" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
       <c r="L18" s="8"/>
     </row>
-    <row r="19" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="9">
         <v>0.375</v>
       </c>
@@ -1352,17 +1346,17 @@
       <c r="C19" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
       <c r="L19" s="8"/>
     </row>
-    <row r="20" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20" s="9">
         <v>0.39583333333333331</v>
       </c>
@@ -1372,17 +1366,17 @@
       <c r="C20" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
       <c r="L20" s="8"/>
     </row>
-    <row r="21" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A21" s="9">
         <v>0.41666666666666669</v>
       </c>
@@ -1392,17 +1386,17 @@
       <c r="C21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A22" s="9">
         <v>0.4375</v>
       </c>
@@ -1412,17 +1406,17 @@
       <c r="C22" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A23" s="9">
         <v>0.45833333333333331</v>
       </c>
@@ -1432,17 +1426,17 @@
       <c r="C23" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A24" s="9">
         <v>0.47916666666666669</v>
       </c>
@@ -1452,17 +1446,17 @@
       <c r="C24" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A25" s="9">
         <v>0.5</v>
       </c>
@@ -1472,19 +1466,19 @@
       <c r="C25" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
       <c r="L25" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="9">
         <v>0.5</v>
       </c>
@@ -1494,19 +1488,19 @@
       <c r="C26" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
       <c r="L26" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A27" s="9">
         <v>0.52083333333333337</v>
       </c>
@@ -1516,17 +1510,17 @@
       <c r="C27" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A28" s="9">
         <v>0.54166666666666663</v>
       </c>
@@ -1536,17 +1530,17 @@
       <c r="C28" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A29" s="9">
         <v>0.5625</v>
       </c>
@@ -1556,17 +1550,17 @@
       <c r="C29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
       <c r="L29" s="8"/>
     </row>
-    <row r="30" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="9">
         <v>0.58333333333333337</v>
       </c>
@@ -1576,17 +1570,17 @@
       <c r="C30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="15"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:12" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A31" s="9">
         <v>0.60416666666666663</v>
       </c>
@@ -1596,59 +1590,59 @@
       <c r="C31" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" ht="35.049999999999997" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:12" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="A32" s="9"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="12"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
-      <c r="L32" s="12"/>
-    </row>
-    <row r="33" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D32" s="10"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+    </row>
+    <row r="33" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
-      <c r="L33" s="12"/>
-    </row>
-    <row r="34" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D33" s="10"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+    </row>
+    <row r="34" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="9"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-    </row>
-    <row r="35" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D34" s="10"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+    </row>
+    <row r="35" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="9"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -1662,7 +1656,7 @@
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="9"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -1676,7 +1670,7 @@
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="9"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -1690,7 +1684,7 @@
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="9"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -1704,7 +1698,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="9"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -1718,7 +1712,7 @@
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="9"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -1732,7 +1726,7 @@
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="9"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -1746,7 +1740,7 @@
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
     </row>
-    <row r="42" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="9"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -1760,7 +1754,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="9"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -1774,7 +1768,7 @@
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="9"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -1788,7 +1782,7 @@
       <c r="K44" s="8"/>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="9"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -1802,7 +1796,7 @@
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="9"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -1816,7 +1810,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="9"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -1830,7 +1824,7 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="9"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -1844,7 +1838,7 @@
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
     </row>
-    <row r="49" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="9"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -1858,7 +1852,7 @@
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -1872,7 +1866,7 @@
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -1886,7 +1880,7 @@
       <c r="K51" s="8"/>
       <c r="L51" s="8"/>
     </row>
-    <row r="52" spans="1:12" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -1901,7 +1895,7 @@
       <c r="L52" s="8"/>
     </row>
   </sheetData>
-  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="87" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;CGrading sheet for IDMA oral exam June 2026: Page &amp;P of &amp;N</oddFooter>

</xml_diff>